<commit_message>
added utility bill script and activity log scripts
</commit_message>
<xml_diff>
--- a/Excel-files/Customer_List.xlsx
+++ b/Excel-files/Customer_List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BS01503\Documents\load testing Script-BSS\Excel-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25FA3CAE-F26A-459D-B913-A420A480C1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BC61489-1ECB-4B5F-A66C-8A4CE5124970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="-40" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Management" sheetId="1" r:id="rId1"/>
@@ -20,39 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
     <t>SID</t>
-  </si>
-  <si>
-    <t>SID2609001228</t>
-  </si>
-  <si>
-    <t>SID2609001227</t>
-  </si>
-  <si>
-    <t>SID2609001226</t>
-  </si>
-  <si>
-    <t>SID2609001225</t>
-  </si>
-  <si>
-    <t>SID2609001224</t>
-  </si>
-  <si>
-    <t>SID2609001223</t>
-  </si>
-  <si>
-    <t>SID2609001222</t>
-  </si>
-  <si>
-    <t>SID2609001221</t>
-  </si>
-  <si>
-    <t>SID2609001220</t>
-  </si>
-  <si>
-    <t>SID2609001219</t>
   </si>
 </sst>
 </file>
@@ -122,7 +92,46 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -136,12 +145,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MyTable" displayName="MyTable" ref="A1:A11" totalsRowShown="0">
-  <autoFilter ref="A1:A11" xr:uid="{00000000-0009-0000-0100-000001000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MyTable" displayName="MyTable" ref="A1:A2" insertRow="1" totalsRowShown="0" dataDxfId="0">
+  <autoFilter ref="A1:A2" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SID" totalsRowLabel="Total"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SID" totalsRowLabel="Total" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -435,7 +444,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20" style="2" bestFit="1" customWidth="1"/>
@@ -447,54 +456,7 @@
       </c>
     </row>
     <row r="2" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>10</v>
-      </c>
+      <c r="A2" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>